<commit_message>
Simulación: bloque de chequeos de consistencia con los números de la hoja (cobranza 100 %, comisiones acotadas, conversión a venta > 0, cadena decreciente) integrado al estado; verificación con cobranza > 100 %
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/simuladores/01_Simulacion_Embudo_Low_Ticket_Bumps_Upsells.xlsx
+++ b/excel/simuladores/01_Simulacion_Embudo_Low_Ticket_Bumps_Upsells.xlsx
@@ -110,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,6 +149,7 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -955,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -992,12 +993,12 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>IF(AND(ISNUMBER(C7),C7&gt;=0,ISNUMBER(C9),C9&gt;=0,ISNUMBER(C11),C11&gt;=0,C11&lt;=1,ISNUMBER(C13),C13&gt;=0,C13&lt;=1,ISNUMBER(C18),C18&gt;=0,ISNUMBER(C20),C20&gt;=0,C20&lt;=1,ISNUMBER(C22),C22&gt;=0,ISNUMBER(C24),C24&gt;=0,C24&lt;=1,ISNUMBER(C26),C26&gt;=0,ISNUMBER(C28),C28&gt;=0,C28&lt;=1,ISNUMBER(C30),C30&gt;=0,ISNUMBER(C32),C32&gt;=0,C32&lt;=1,ISNUMBER(C34),C34&gt;=0,ISNUMBER(C36),C36&gt;=0,C36&lt;=1,ISNUMBER(C38),C38&gt;=0,ISNUMBER(C40),C40&gt;=0,C40&lt;=1,ISNUMBER(C42),C42&gt;=0,ISNUMBER(C44),C44&gt;=0,C44&lt;=1,ISNUMBER(C46),C46&gt;=0,ISNUMBER(C54),C54&gt;=0,C54&lt;=1,ISNUMBER(C55),C55&gt;=0,C55&lt;=1,ISNUMBER(C56),C56&gt;=0,C56&lt;=1,ISNUMBER(C59),C59&gt;=0,C59&lt;=1,ISNUMBER(C60),C60&gt;=0,C60&lt;=1,ISNUMBER(C62),C62&gt;=0,C62&lt;=1,ISNUMBER(C65),C65&gt;=0,ISNUMBER(C67),C67&gt;=0,ISNUMBER(C72),C72&gt;=0,ISNUMBER(C77),C77&gt;=0,C77&lt;=1,ISNUMBER(C86),C86&gt;=0),"OK","REVISAR")</f>
+        <f>IF(AND(ISNUMBER(C7),C7&gt;=0,ISNUMBER(C9),C9&gt;=0,ISNUMBER(C11),C11&gt;=0,C11&lt;=1,ISNUMBER(C13),C13&gt;=0,C13&lt;=1,ISNUMBER(C18),C18&gt;=0,ISNUMBER(C20),C20&gt;=0,C20&lt;=1,ISNUMBER(C22),C22&gt;=0,ISNUMBER(C24),C24&gt;=0,C24&lt;=1,ISNUMBER(C26),C26&gt;=0,ISNUMBER(C28),C28&gt;=0,C28&lt;=1,ISNUMBER(C30),C30&gt;=0,ISNUMBER(C32),C32&gt;=0,C32&lt;=1,ISNUMBER(C34),C34&gt;=0,ISNUMBER(C36),C36&gt;=0,C36&lt;=1,ISNUMBER(C38),C38&gt;=0,ISNUMBER(C40),C40&gt;=0,C40&lt;=1,ISNUMBER(C42),C42&gt;=0,ISNUMBER(C44),C44&gt;=0,C44&lt;=1,ISNUMBER(C46),C46&gt;=0,ISNUMBER(C54),C54&gt;=0,C54&lt;=1,ISNUMBER(C55),C55&gt;=0,C55&lt;=1,ISNUMBER(C56),C56&gt;=0,C56&lt;=1,ISNUMBER(C59),C59&gt;=0,C59&lt;=1,ISNUMBER(C60),C60&gt;=0,C60&lt;=1,ISNUMBER(C62),C62&gt;=0,C62&lt;=1,ISNUMBER(C65),C65&gt;=0,ISNUMBER(C67),C67&gt;=0,ISNUMBER(C72),C72&gt;=0,ISNUMBER(C77),C77&gt;=0,C77&lt;=1,ISNUMBER(C86),C86&gt;=0,COUNTIF(C95:C102,"REVISAR")=0),"OK","REVISAR")</f>
         <v/>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>OK = todos los supuestos tienen sentido. REVISAR = hay un porcentaje fuera de 0 a 1, un negativo o un texto donde va un número.</t>
+          <t>OK = todos los supuestos tienen sentido y los chequeos del final pasan. REVISAR = hay un porcentaje fuera de 0 a 1, un negativo, un texto donde va un número, o un chequeo de consistencia que falla (mirá el bloque Chequeos al final).</t>
         </is>
       </c>
     </row>
@@ -2354,22 +2355,151 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="32" customHeight="1">
-      <c r="B95" s="5" t="inlineStr">
+    <row r="94">
+      <c r="B94" s="13" t="inlineStr">
+        <is>
+          <t>Chequeos: tus números tienen que ser consistentes, no solo estar en rango</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="n"/>
+      <c r="D94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Los supuestos de tráfico son mayores a cero</t>
+        </is>
+      </c>
+      <c r="C95" s="34">
+        <f>IF(AND($C$7&gt;0,$C$11&gt;0,$C$13&gt;0),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>Con un 0 en el tráfico o en la conversión de la página no hay unidades y el modelo no dice nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>La curva de cobranza suma 100 %</t>
+        </is>
+      </c>
+      <c r="C96" s="34">
+        <f>IF(ABS($C$54+$C$55+$C$56-1)&lt;0.001,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>Supuestos → cobranza mes 1 + mes 2 + mes 3 = 100 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Comisiones + reembolsos menores al 60 %</t>
+        </is>
+      </c>
+      <c r="C97" s="34">
+        <f>IF(($C$59+$C$60+$C$62)&lt;0.6,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>Si suman más, revisá los porcentajes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>La inversión es mayor a cero</t>
+        </is>
+      </c>
+      <c r="C98" s="34">
+        <f>IF($C$9&gt;0,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D98" s="5" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>La meta de ventas es alcanzable (hay conversión a venta)</t>
+        </is>
+      </c>
+      <c r="C99" s="34">
+        <f>IF($C$15&gt;0,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>Con conversión a venta en 0, la inversión para la meta dice 'inalcanzable con estos supuestos'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Las conversiones están entre 0 y 100 %</t>
+        </is>
+      </c>
+      <c r="C100" s="34">
+        <f>IF(AND($C$11&gt;=0,$C$11&lt;=1,$C$13&gt;=0,$C$13&lt;=1,$C$20&gt;=0,$C$20&lt;=1,$C$24&gt;=0,$C$24&lt;=1,$C$28&gt;=0,$C$28&lt;=1,$C$32&gt;=0,$C$32&lt;=1,$C$36&gt;=0,$C$36&lt;=1,$C$40&gt;=0,$C$40&lt;=1,$C$44&gt;=0,$C$44&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Un 25 % se escribe 25 % (o 0,25), no 25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>El margen de seguridad está entre 0 y 100 %</t>
+        </is>
+      </c>
+      <c r="C101" s="34">
+        <f>IF(AND($C$77&gt;=0,$C$77&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D101" s="5" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>La cadena es decreciente (cada etapa tiene menos gente que la anterior)</t>
+        </is>
+      </c>
+      <c r="C102" s="34">
+        <f>IF(AND($C$12&lt;=$C$10,$C$14&lt;=$C$12),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>Si falla, alguna conversión está por encima de 100 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="32" customHeight="1">
+      <c r="B104" s="5" t="inlineStr">
         <is>
           <t>Cómo se usa: cambiá cualquier celda amarilla (inversión, CPM, CTR, conversión de la landing, show, solicitudes, cierre, precios, comisiones, costos, cobranza, meta) y mirá cómo se mueven todas las celdas azules de abajo: cantidades, costos por paso, facturado, cash neto, ganancia, ROAS, el techo y el objetivo, el semáforo y la inversión para tu meta.</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="32" customHeight="1">
-      <c r="B96" s="5" t="inlineStr">
+    <row r="105" ht="32" customHeight="1">
+      <c r="B105" s="5" t="inlineStr">
         <is>
           <t>Una variable por vez. Si querés comparar dos ideas, duplicá la hoja (clic derecho en la pestaña → Duplicar) y cambiá en cada copia una sola cosa.</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="32" customHeight="1">
-      <c r="B97" s="5" t="inlineStr">
+    <row r="106" ht="32" customHeight="1">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>Para volver al ejemplo, el valor original de cada supuesto está en la hoja Inicio.</t>
         </is>
@@ -2377,11 +2507,11 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B96:D96"/>
-    <mergeCell ref="B97:D97"/>
-    <mergeCell ref="B95:D95"/>
+    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="B105:D105"/>
+    <mergeCell ref="B106:D106"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4">
+  <conditionalFormatting sqref="C95:C102">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -2389,25 +2519,33 @@
       <formula>"REVISAR"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C4">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"REVISAR"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C73">
-    <cfRule type="expression" priority="3" dxfId="0">
+    <cfRule type="expression" priority="5" dxfId="0">
       <formula>LEFT(C73,5)="VERDE"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="2">
+    <cfRule type="expression" priority="6" dxfId="2">
       <formula>LEFT(C73,8)="AMARILLO"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="1">
+    <cfRule type="expression" priority="7" dxfId="1">
       <formula>LEFT(C73,4)="ROJO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C85">
-    <cfRule type="expression" priority="6" dxfId="0">
+    <cfRule type="expression" priority="8" dxfId="0">
       <formula>LEFT(C85,5)="VERDE"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="2">
+    <cfRule type="expression" priority="9" dxfId="2">
       <formula>LEFT(C85,8)="AMARILLO"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
+    <cfRule type="expression" priority="10" dxfId="1">
       <formula>LEFT(C85,4)="ROJO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>